<commit_message>
Improve car approach and search rotation
</commit_message>
<xml_diff>
--- a/daily_work/2026-06-04_daily_work.xlsx
+++ b/daily_work/2026-06-04_daily_work.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日计划表" sheetId="1" r:id="Rfc6c10f56ff74a0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日计划表" sheetId="1" r:id="Recd8f019d84e4fe2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -534,7 +534,7 @@
         <x:v>待补充</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="36" customHeight="1">
+    <x:row r="11" ht="96" customHeight="1">
       <x:c r="A11" s="3" t="str">
         <x:v>10</x:v>
       </x:c>
@@ -548,16 +548,20 @@
         <x:v>搜房一直顺时针，撞墙/门第 6 次后应切逆时针</x:v>
       </x:c>
       <x:c r="E11" s="3" t="str">
-        <x:v>增加顺/逆时针状态切换；第 6 次撞墙/门后改为左转视野并右上滑</x:v>
+        <x:v>增加顺/逆时针状态切换；第 6 次撞墙/门后改为左转视野并右上滑；出房找出口绕圈同步接入方向切换</x:v>
       </x:c>
       <x:c r="F11" s="3" t="str">
-        <x:v>室内专项验证一圈后是否切换方向，避免持续顺时针卡墙</x:v>
+        <x:v>室内专项验证一圈后是否切换方向，避免持续顺时针卡墙；出房专项验证找出口绕圈是否能反向</x:v>
       </x:c>
       <x:c r="G11" s="3" t="str">
-        <x:v>待开始</x:v>
+        <x:v>代码完成，待专项验证</x:v>
       </x:c>
       <x:c r="H11" s="3" t="str">
-        <x:v>待补充</x:v>
+        <x:v>1. 定位室内搜房绕圈的 `wall_hit_count` 原来只按连续撞墙/门计数，补转后识别回 `indoor` 会被清零，导致难以触发第 6 次切换。
+2. 将室内搜房绕圈改为累计撞墙/门计数，第 6 次后从 `left_up` 切到 `right_up`，并改为向左补转。
+3. 抽出 `move_mode` 方向辅助逻辑，统一计算左上/右上滑动和对应补转方向。
+4. 出房找出口绕圈原来固定左上滑动加右转视角，已改为 `left_up/right_up` 状态机。
+5. 出房找出口阶段同样累计撞墙/门，第 6 次后切到反向绕圈，避免一直顺时针卡墙。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="123" customHeight="1">
@@ -619,7 +623,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R444ad22b5b944e57"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb272a2a63b5420b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>